<commit_message>
Le bases no rodape dos holerites (payroll-02 e payroll-03)
Rodape com varios pares rotulo/valor na mesma linha fisica agora vira bases:
nova funcao separarPares + classificacao linha a linha, sem travar a fronteira
(preserva o payroll-02, que tem dois demonstrativos por pagina). +4 testes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saidas/payroll-03.xlsx
+++ b/saidas/payroll-03.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
   <si>
     <t>Pág.</t>
   </si>
@@ -49,36 +49,12 @@
     <t>Conv. Odonto. (S. Franc.)</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Líqüido</t>
-  </si>
-  <si>
-    <t>Base I.N.S.S. :                    1.967,07              F.G.T.S. do Mês</t>
-  </si>
-  <si>
-    <t>Base I.N.S.S. :                    1.975,31              F.G.T.S. do Mês</t>
-  </si>
-  <si>
     <t>/337 Diferença de 13º salário</t>
   </si>
   <si>
     <t>/303 Trib.INSS (13o)</t>
   </si>
   <si>
-    <t>Base I.N.S.S. :                    1.978,83              F.G.T.S. do Mês</t>
-  </si>
-  <si>
-    <t>Base I.R.R.F. :                    1.779,77              Base I.R.R.F. 13o</t>
-  </si>
-  <si>
-    <t>Base I.N.S.S. :                    1.933,43              F.G.T.S. do Mês</t>
-  </si>
-  <si>
-    <t>Base I.N.S.S. :                    1.810,19              F.G.T.S. do Mês</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -115,15 +91,6 @@
     <t>10,99</t>
   </si>
   <si>
-    <t>859,46</t>
-  </si>
-  <si>
-    <t>1.107,61</t>
-  </si>
-  <si>
-    <t>157,37</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -148,15 +115,6 @@
     <t>177,77</t>
   </si>
   <si>
-    <t>860,20</t>
-  </si>
-  <si>
-    <t>1.115,11</t>
-  </si>
-  <si>
-    <t>158,02</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
@@ -178,24 +136,12 @@
     <t>176,02</t>
   </si>
   <si>
-    <t>860,29</t>
-  </si>
-  <si>
-    <t>1.118,54</t>
-  </si>
-  <si>
     <t>23,04</t>
   </si>
   <si>
     <t>1,84</t>
   </si>
   <si>
-    <t>158,30</t>
-  </si>
-  <si>
-    <t>21,20</t>
-  </si>
-  <si>
     <t>4</t>
   </si>
   <si>
@@ -220,15 +166,6 @@
     <t>174,00</t>
   </si>
   <si>
-    <t>856,43</t>
-  </si>
-  <si>
-    <t>1.077,00</t>
-  </si>
-  <si>
-    <t>154,67</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -242,15 +179,6 @@
   </si>
   <si>
     <t>144,81</t>
-  </si>
-  <si>
-    <t>827,24</t>
-  </si>
-  <si>
-    <t>982,95</t>
-  </si>
-  <si>
-    <t>144,82</t>
   </si>
 </sst>
 </file>
@@ -637,13 +565,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="22" width="14" customWidth="1"/>
+    <col min="1" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -686,369 +614,225 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="C2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="E2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="F2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="G2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="H2" t="s">
         <v>21</v>
       </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" t="s">
         <v>24</v>
       </c>
-      <c r="D2" t="s">
+      <c r="L3" t="s">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>34</v>
       </c>
-      <c r="N2" t="s">
+      <c r="B4" t="s">
         <v>35</v>
       </c>
-      <c r="O2" t="s">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
         <v>36</v>
       </c>
-      <c r="P2" t="s">
+      <c r="G4" t="s">
         <v>37</v>
       </c>
-      <c r="Q2" t="s">
-        <v>37</v>
-      </c>
-      <c r="R2" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
-      <c r="T2" t="s">
-        <v>37</v>
-      </c>
-      <c r="U2" t="s">
-        <v>37</v>
-      </c>
-      <c r="V2" t="s">
-        <v>37</v>
+      <c r="H4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N4" t="s">
+        <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="L5" t="s">
         <v>25</v>
       </c>
-      <c r="E3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" t="s">
-        <v>44</v>
-      </c>
-      <c r="K3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="M5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
         <v>45</v>
       </c>
-      <c r="N3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>37</v>
-      </c>
-      <c r="R3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S3" t="s">
-        <v>37</v>
-      </c>
-      <c r="T3" t="s">
-        <v>37</v>
-      </c>
-      <c r="U3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
+      <c r="L6" t="s">
         <v>25</v>
       </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" t="s">
-        <v>51</v>
-      </c>
-      <c r="H4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I4" t="s">
-        <v>53</v>
-      </c>
-      <c r="J4" t="s">
-        <v>54</v>
-      </c>
-      <c r="K4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M4" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" t="s">
-        <v>56</v>
-      </c>
-      <c r="O4" t="s">
-        <v>37</v>
-      </c>
-      <c r="P4" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>57</v>
-      </c>
-      <c r="R4" t="s">
-        <v>58</v>
-      </c>
-      <c r="S4" t="s">
-        <v>59</v>
-      </c>
-      <c r="T4" t="s">
-        <v>60</v>
-      </c>
-      <c r="U4" t="s">
-        <v>37</v>
-      </c>
-      <c r="V4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" t="s">
-        <v>65</v>
-      </c>
-      <c r="H5" t="s">
-        <v>66</v>
-      </c>
-      <c r="I5" t="s">
-        <v>67</v>
-      </c>
-      <c r="J5" t="s">
-        <v>68</v>
-      </c>
-      <c r="K5" t="s">
-        <v>32</v>
-      </c>
-      <c r="L5" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" t="s">
-        <v>69</v>
-      </c>
-      <c r="N5" t="s">
-        <v>70</v>
-      </c>
-      <c r="O5" t="s">
-        <v>37</v>
-      </c>
-      <c r="P5" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R5" t="s">
-        <v>37</v>
-      </c>
-      <c r="S5" t="s">
-        <v>37</v>
-      </c>
-      <c r="T5" t="s">
-        <v>37</v>
-      </c>
-      <c r="U5" t="s">
-        <v>71</v>
-      </c>
-      <c r="V5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" t="s">
-        <v>74</v>
-      </c>
-      <c r="H6" t="s">
-        <v>75</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>76</v>
-      </c>
-      <c r="K6" t="s">
-        <v>32</v>
-      </c>
-      <c r="L6" t="s">
-        <v>33</v>
-      </c>
       <c r="M6" t="s">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="N6" t="s">
-        <v>78</v>
-      </c>
-      <c r="O6" t="s">
-        <v>37</v>
-      </c>
-      <c r="P6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>37</v>
-      </c>
-      <c r="R6" t="s">
-        <v>37</v>
-      </c>
-      <c r="S6" t="s">
-        <v>37</v>
-      </c>
-      <c r="T6" t="s">
-        <v>37</v>
-      </c>
-      <c r="U6" t="s">
-        <v>37</v>
-      </c>
-      <c r="V6" t="s">
-        <v>79</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>